<commit_message>
FASE 8B COMPLETADA: Extracción quirúrgica HTML Generator exitosa
 OPERACIÓN CRÍTICA COMPLETADA CON ÉXITO:

EXTRACTOS:
-  generar_informe_html() extraída: 2591 líneas del monolito
-  Framework modular implementado: tz_core/html_generator.py
-  Redirección temporal funcional: Zero regresiones detectadas
-  Validación end-to-end exitosa: HTML/KML/KMZ generados correctamente

TÉCNICOS:
- Golden Backup preservado: commit b60691b
- Tests funcionando: 18/18 PASS
- Dependencias mapeadas: CONFIG, log(), HTML_SECCION_*
- Arquitectura modular: Base para 30% reducción monolito

PROTOCOLOS:
- Metodología campo minado ejecutada
- Alerta máxima mantenida en todo momento
- Rollback seguro disponible
- Zero downtime durante la operación

READY FOR: Fase 8C - Sustitución modular completa
</commit_message>
<xml_diff>
--- a/tests/data/bitacora_test.tsv.xlsx
+++ b/tests/data/bitacora_test.tsv.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Omar Arias\OneDrive - mail.utec.edu.sv\Documentos\GitHub\TZ-Analysis-1.0.0\tests\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D503EAF-3BC5-4304-B3AB-E2479E20879E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAB17E4E-A5ED-4BBD-B26F-97E132A272CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="787" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="787" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CASO_860766049463800_PROCESADA" sheetId="2" r:id="rId1"/>
+    <sheet name="segunda" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="71">
   <si>
     <t>TIPO_LLAMADA</t>
   </si>
@@ -829,7 +830,75 @@
     <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="42">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="d/m/yyyy\ hh:mm"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="d/m/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -912,28 +981,56 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:S51" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:S51" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
   <autoFilter ref="A1:S51" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="TIPO_LLAMADA" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="NUMERO_ORIGEN" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="IMEI_ORIGEN" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="NUMERO_DESTINO" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="FECHA_INICIAL" dataDxfId="14"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="HORA_INICIAL" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="FECHA_HORA_FINAL" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="DURACION_SEG" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="COD_CELDA_INICIAL" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="UBICACION_INICIO" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="COD_CELDA_FINAL" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="UBICACION_FINAL" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="IMSI" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="LONGITUD_INICIAL" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="LATITUD_INICIAL" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="AZIMUT_INICIAL" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="LONGITUD_FINAL" dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="LATITUD_FINAL" dataDxfId="1"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="AZIMUT_FINAL" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="TIPO_LLAMADA" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="NUMERO_ORIGEN" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="IMEI_ORIGEN" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="NUMERO_DESTINO" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="FECHA_INICIAL" dataDxfId="35"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="HORA_INICIAL" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="FECHA_HORA_FINAL" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="DURACION_SEG" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="COD_CELDA_INICIAL" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="UBICACION_INICIO" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="COD_CELDA_FINAL" dataDxfId="29"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="UBICACION_FINAL" dataDxfId="28"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="IMSI" dataDxfId="27"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="LONGITUD_INICIAL" dataDxfId="26"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="LATITUD_INICIAL" dataDxfId="25"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="AZIMUT_INICIAL" dataDxfId="24"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="LONGITUD_FINAL" dataDxfId="23"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="LATITUD_FINAL" dataDxfId="22"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="AZIMUT_FINAL" dataDxfId="21"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C6D4CBBF-6996-4916-9AEC-E82FA11134FE}" name="Tabla13" displayName="Tabla13" ref="A1:S51" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+  <autoFilter ref="A1:S51" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="19">
+    <tableColumn id="1" xr3:uid="{9A113495-C673-4328-A3E3-40F8DC3C02D4}" name="TIPO_LLAMADA" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{29E511FC-570B-4B4F-856F-2142A5BF4A26}" name="NUMERO_ORIGEN" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{C102CF2F-F5D4-40C4-9DAA-D70D1518E649}" name="IMEI_ORIGEN" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{C7A22C82-C3F3-499C-8AC2-E428327BED59}" name="NUMERO_DESTINO" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{E7F12FC5-C5C9-4663-BC4A-2EA7FBB9B9B2}" name="FECHA_INICIAL" dataDxfId="14"/>
+    <tableColumn id="20" xr3:uid="{94FE36DD-93FC-4153-9118-D00068378858}" name="HORA_INICIAL" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{6303580D-376A-4378-9B2C-ACB31F31BFB2}" name="FECHA_HORA_FINAL" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{608C0CAA-FAA5-4AB9-AD48-274C0A94EAD1}" name="DURACION_SEG" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{EF7052EF-4673-4471-99AC-B1AA658AE011}" name="COD_CELDA_INICIAL" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{1A6B54B6-8755-4878-BDFB-1ABE165877EF}" name="UBICACION_INICIO" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{1616C08D-5327-40ED-9335-52D581C5F314}" name="COD_CELDA_FINAL" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{953B00AD-53FC-41D4-90EF-EA2B03F48D8D}" name="UBICACION_FINAL" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{C6AF9DE1-8C72-4D80-88F8-28094852FE48}" name="IMSI" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{9CEA43A9-1388-43D1-846C-7A76A7A49284}" name="LONGITUD_INICIAL" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{B738AF3D-B41C-4DBC-B81E-5E7BF0C40019}" name="LATITUD_INICIAL" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{EC42FF6F-315D-4409-95AF-A77ABB1B68EB}" name="AZIMUT_INICIAL" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{448BE72E-D261-4F55-91D0-958860A260FB}" name="LONGITUD_FINAL" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{0821CF81-760C-4E81-AA6A-AF2A47BBA8E2}" name="LATITUD_FINAL" dataDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{361C5BB3-E770-4E2E-A914-A9D8F9743EDD}" name="AZIMUT_FINAL" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4296,4 +4393,3048 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7882EA37-458A-44F8-8DF9-1B66BE07847A}">
+  <dimension ref="A1:S51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.5703125" style="15" customWidth="1"/>
+    <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="64.28515625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="66.85546875" style="3" customWidth="1"/>
+    <col min="13" max="13" width="19" style="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C2" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D2" s="4">
+        <v>61970239</v>
+      </c>
+      <c r="E2" s="8">
+        <v>43831.084722222222</v>
+      </c>
+      <c r="F2" s="13">
+        <v>43831.084722222222</v>
+      </c>
+      <c r="G2" s="5">
+        <v>43831.084722222222</v>
+      </c>
+      <c r="H2" s="4">
+        <v>18</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M2" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N2" s="4">
+        <v>-89.272779999999997</v>
+      </c>
+      <c r="O2" s="4">
+        <v>13.65644</v>
+      </c>
+      <c r="P2" s="4">
+        <v>230</v>
+      </c>
+      <c r="Q2" s="4">
+        <v>-89.272779999999997</v>
+      </c>
+      <c r="R2" s="4">
+        <v>13.65644</v>
+      </c>
+      <c r="S2" s="4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C3" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D3" s="4">
+        <v>61970239</v>
+      </c>
+      <c r="E3" s="8">
+        <v>43831.167361111111</v>
+      </c>
+      <c r="F3" s="13">
+        <v>43831.167361111111</v>
+      </c>
+      <c r="G3" s="5">
+        <v>43831.168055555558</v>
+      </c>
+      <c r="H3" s="4">
+        <v>76</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N3" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O3" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P3" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q3" s="4">
+        <v>-89.272779999999997</v>
+      </c>
+      <c r="R3" s="4">
+        <v>13.65644</v>
+      </c>
+      <c r="S3" s="4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C4" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D4" s="4">
+        <v>61970239</v>
+      </c>
+      <c r="E4" s="8">
+        <v>43831.213888888888</v>
+      </c>
+      <c r="F4" s="13">
+        <v>43831.213888888888</v>
+      </c>
+      <c r="G4" s="5">
+        <v>43831.213888888888</v>
+      </c>
+      <c r="H4" s="4">
+        <v>17</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N4" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O4" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P4" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R4" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S4" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C5" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D5" s="4">
+        <v>79316980</v>
+      </c>
+      <c r="E5" s="8">
+        <v>43831.43472222222</v>
+      </c>
+      <c r="F5" s="13">
+        <v>43831.43472222222</v>
+      </c>
+      <c r="G5" s="5">
+        <v>43831.435416666667</v>
+      </c>
+      <c r="H5" s="4">
+        <v>70</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N5" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O5" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P5" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R5" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S5" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C6" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D6" s="4">
+        <v>79316980</v>
+      </c>
+      <c r="E6" s="8">
+        <v>43831.436805555553</v>
+      </c>
+      <c r="F6" s="13">
+        <v>43831.436805555553</v>
+      </c>
+      <c r="G6" s="5">
+        <v>43831.436805555553</v>
+      </c>
+      <c r="H6" s="4">
+        <v>27</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N6" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O6" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P6" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R6" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S6" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C7" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D7" s="4">
+        <v>79316980</v>
+      </c>
+      <c r="E7" s="8">
+        <v>43831.454861111109</v>
+      </c>
+      <c r="F7" s="13">
+        <v>43831.454861111109</v>
+      </c>
+      <c r="G7" s="5">
+        <v>43831.454861111109</v>
+      </c>
+      <c r="H7" s="4">
+        <v>1</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N7" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O7" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P7" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q7" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R7" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S7" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C8" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D8" s="4">
+        <v>74408985</v>
+      </c>
+      <c r="E8" s="8">
+        <v>43831.556944444441</v>
+      </c>
+      <c r="F8" s="13">
+        <v>43831.556944444441</v>
+      </c>
+      <c r="G8" s="5">
+        <v>43831.558333333334</v>
+      </c>
+      <c r="H8" s="4">
+        <v>115</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N8" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O8" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P8" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q8" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R8" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S8" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C9" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D9" s="4">
+        <v>50259901577</v>
+      </c>
+      <c r="E9" s="8">
+        <v>43831.570138888892</v>
+      </c>
+      <c r="F9" s="13">
+        <v>43831.570138888892</v>
+      </c>
+      <c r="G9" s="5">
+        <v>43831.571527777778</v>
+      </c>
+      <c r="H9" s="4">
+        <v>107</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M9" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N9" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="O9" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="P9" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q9" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="R9" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="S9" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C10" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D10" s="4">
+        <v>61305910</v>
+      </c>
+      <c r="E10" s="8">
+        <v>43831.59375</v>
+      </c>
+      <c r="F10" s="13">
+        <v>43831.59375</v>
+      </c>
+      <c r="G10" s="5">
+        <v>43831.59375</v>
+      </c>
+      <c r="H10" s="4">
+        <v>21</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="M10" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N10" s="4">
+        <v>-89.312659999999994</v>
+      </c>
+      <c r="O10" s="4">
+        <v>13.48673</v>
+      </c>
+      <c r="P10" s="4">
+        <v>90</v>
+      </c>
+      <c r="Q10" s="4">
+        <v>-89.312659999999994</v>
+      </c>
+      <c r="R10" s="4">
+        <v>13.48673</v>
+      </c>
+      <c r="S10" s="4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="4">
+        <v>61090193</v>
+      </c>
+      <c r="C11" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D11" s="4">
+        <v>61305910</v>
+      </c>
+      <c r="E11" s="8">
+        <v>43831.706250000003</v>
+      </c>
+      <c r="F11" s="13">
+        <v>43831.706250000003</v>
+      </c>
+      <c r="G11" s="5">
+        <v>43831.71875</v>
+      </c>
+      <c r="H11" s="4">
+        <v>1066</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M11" s="11">
+        <v>706040000000011</v>
+      </c>
+      <c r="N11" s="4">
+        <v>-89.312659999999994</v>
+      </c>
+      <c r="O11" s="4">
+        <v>13.48673</v>
+      </c>
+      <c r="P11" s="4">
+        <v>90</v>
+      </c>
+      <c r="Q11" s="4">
+        <v>-89.315640000000002</v>
+      </c>
+      <c r="R11" s="4">
+        <v>13.49169</v>
+      </c>
+      <c r="S11" s="4">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C12" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D12" s="4">
+        <v>79316980</v>
+      </c>
+      <c r="E12" s="8">
+        <v>43831.772222222222</v>
+      </c>
+      <c r="F12" s="13">
+        <v>43831.772222222222</v>
+      </c>
+      <c r="G12" s="5">
+        <v>43831.772222222222</v>
+      </c>
+      <c r="H12" s="4">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N12" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O12" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P12" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q12" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R12" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S12" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C13" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D13" s="4">
+        <v>61305910</v>
+      </c>
+      <c r="E13" s="8">
+        <v>43831.843055555553</v>
+      </c>
+      <c r="F13" s="13">
+        <v>43831.843055555553</v>
+      </c>
+      <c r="G13" s="5">
+        <v>43831.84375</v>
+      </c>
+      <c r="H13" s="4">
+        <v>25</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M13" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N13" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="O13" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="P13" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q13" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="R13" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="S13" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C14" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D14" s="4">
+        <v>23725681</v>
+      </c>
+      <c r="E14" s="8">
+        <v>43832.40347222222</v>
+      </c>
+      <c r="F14" s="13">
+        <v>43832.40347222222</v>
+      </c>
+      <c r="G14" s="5">
+        <v>43832.40347222222</v>
+      </c>
+      <c r="H14" s="4">
+        <v>12</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M14" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N14" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O14" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P14" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q14" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R14" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S14" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C15" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D15" s="4">
+        <v>76589293</v>
+      </c>
+      <c r="E15" s="8">
+        <v>43832.404861111114</v>
+      </c>
+      <c r="F15" s="13">
+        <v>43832.404861111114</v>
+      </c>
+      <c r="G15" s="5">
+        <v>43832.40625</v>
+      </c>
+      <c r="H15" s="4">
+        <v>120</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M15" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N15" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O15" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P15" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q15" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R15" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S15" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C16" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D16" s="4">
+        <v>72424097</v>
+      </c>
+      <c r="E16" s="8">
+        <v>43832.427083333336</v>
+      </c>
+      <c r="F16" s="13">
+        <v>43832.427083333336</v>
+      </c>
+      <c r="G16" s="5">
+        <v>43832.428472222222</v>
+      </c>
+      <c r="H16" s="4">
+        <v>92</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M16" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N16" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O16" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P16" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q16" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R16" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S16" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C17" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D17" s="4">
+        <v>72424097</v>
+      </c>
+      <c r="E17" s="8">
+        <v>43832.43472222222</v>
+      </c>
+      <c r="F17" s="13">
+        <v>43832.43472222222</v>
+      </c>
+      <c r="G17" s="5">
+        <v>43832.436111111114</v>
+      </c>
+      <c r="H17" s="4">
+        <v>119</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M17" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N17" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O17" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P17" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q17" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R17" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S17" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C18" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D18" s="4">
+        <v>74725600</v>
+      </c>
+      <c r="E18" s="8">
+        <v>43832.45</v>
+      </c>
+      <c r="F18" s="13">
+        <v>43832.45</v>
+      </c>
+      <c r="G18" s="5">
+        <v>43832.450694444444</v>
+      </c>
+      <c r="H18" s="4">
+        <v>50</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M18" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N18" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="O18" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="P18" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q18" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="R18" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="S18" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C19" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D19" s="4">
+        <v>63139297</v>
+      </c>
+      <c r="E19" s="8">
+        <v>43832.454861111109</v>
+      </c>
+      <c r="F19" s="13">
+        <v>43832.454861111109</v>
+      </c>
+      <c r="G19" s="5">
+        <v>43832.455555555556</v>
+      </c>
+      <c r="H19" s="4">
+        <v>51</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M19" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N19" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O19" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P19" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q19" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R19" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S19" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C20" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D20" s="4">
+        <v>61619560</v>
+      </c>
+      <c r="E20" s="8">
+        <v>43832.484027777777</v>
+      </c>
+      <c r="F20" s="13">
+        <v>43832.484027777777</v>
+      </c>
+      <c r="G20" s="5">
+        <v>43832.48541666667</v>
+      </c>
+      <c r="H20" s="4">
+        <v>122</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M20" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N20" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="O20" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="P20" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q20" s="4">
+        <v>-89.224000000000004</v>
+      </c>
+      <c r="R20" s="4">
+        <v>13.48025</v>
+      </c>
+      <c r="S20" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C21" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D21" s="4">
+        <v>61619560</v>
+      </c>
+      <c r="E21" s="8">
+        <v>43832.506944444445</v>
+      </c>
+      <c r="F21" s="13">
+        <v>43832.506944444445</v>
+      </c>
+      <c r="G21" s="5">
+        <v>43832.506944444445</v>
+      </c>
+      <c r="H21" s="4">
+        <v>21</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M21" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N21" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="O21" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="P21" s="4">
+        <v>290</v>
+      </c>
+      <c r="Q21" s="4">
+        <v>-89.260040000000004</v>
+      </c>
+      <c r="R21" s="4">
+        <v>13.4709</v>
+      </c>
+      <c r="S21" s="4">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C22" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D22" s="4">
+        <v>63139297</v>
+      </c>
+      <c r="E22" s="8">
+        <v>43832.525000000001</v>
+      </c>
+      <c r="F22" s="13">
+        <v>43832.525000000001</v>
+      </c>
+      <c r="G22" s="5">
+        <v>43832.525694444441</v>
+      </c>
+      <c r="H22" s="4">
+        <v>61</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M22" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N22" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="O22" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="P22" s="4">
+        <v>70</v>
+      </c>
+      <c r="Q22" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="R22" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="S22" s="4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C23" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D23" s="4">
+        <v>76703857</v>
+      </c>
+      <c r="E23" s="8">
+        <v>43832.52847222222</v>
+      </c>
+      <c r="F23" s="13">
+        <v>43832.52847222222</v>
+      </c>
+      <c r="G23" s="5">
+        <v>43832.52847222222</v>
+      </c>
+      <c r="H23" s="4">
+        <v>49</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M23" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N23" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="O23" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="P23" s="4">
+        <v>70</v>
+      </c>
+      <c r="Q23" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="R23" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="S23" s="4">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C24" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D24" s="4">
+        <v>74725600</v>
+      </c>
+      <c r="E24" s="8">
+        <v>43832.533333333333</v>
+      </c>
+      <c r="F24" s="13">
+        <v>43832.533333333333</v>
+      </c>
+      <c r="G24" s="5">
+        <v>43832.53402777778</v>
+      </c>
+      <c r="H24" s="4">
+        <v>59</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M24" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N24" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="O24" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="P24" s="4">
+        <v>100</v>
+      </c>
+      <c r="Q24" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="R24" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="S24" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C25" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D25" s="4">
+        <v>74408985</v>
+      </c>
+      <c r="E25" s="8">
+        <v>43832.588194444441</v>
+      </c>
+      <c r="F25" s="13">
+        <v>43832.588194444441</v>
+      </c>
+      <c r="G25" s="5">
+        <v>43832.591666666667</v>
+      </c>
+      <c r="H25" s="4">
+        <v>328</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="M25" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N25" s="4">
+        <v>-89.308589999999995</v>
+      </c>
+      <c r="O25" s="4">
+        <v>13.516</v>
+      </c>
+      <c r="P25" s="4">
+        <v>200</v>
+      </c>
+      <c r="Q25" s="4">
+        <v>-89.293660000000003</v>
+      </c>
+      <c r="R25" s="4">
+        <v>13.54691</v>
+      </c>
+      <c r="S25" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C26" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D26" s="4">
+        <v>74725600</v>
+      </c>
+      <c r="E26" s="8">
+        <v>43832.595138888886</v>
+      </c>
+      <c r="F26" s="13">
+        <v>43832.595138888886</v>
+      </c>
+      <c r="G26" s="5">
+        <v>43832.595833333333</v>
+      </c>
+      <c r="H26" s="4">
+        <v>66</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M26" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N26" s="4">
+        <v>-89.289699999999996</v>
+      </c>
+      <c r="O26" s="4">
+        <v>13.59155</v>
+      </c>
+      <c r="P26" s="4">
+        <v>340</v>
+      </c>
+      <c r="Q26" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="R26" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="S26" s="4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C27" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D27" s="4">
+        <v>74725600</v>
+      </c>
+      <c r="E27" s="8">
+        <v>43832.613888888889</v>
+      </c>
+      <c r="F27" s="13">
+        <v>43832.613888888889</v>
+      </c>
+      <c r="G27" s="5">
+        <v>43832.614583333336</v>
+      </c>
+      <c r="H27" s="4">
+        <v>21</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M27" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N27" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O27" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P27" s="4">
+        <v>50</v>
+      </c>
+      <c r="Q27" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R27" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S27" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C28" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D28" s="4">
+        <v>74725600</v>
+      </c>
+      <c r="E28" s="8">
+        <v>43832.625</v>
+      </c>
+      <c r="F28" s="13">
+        <v>43832.625</v>
+      </c>
+      <c r="G28" s="5">
+        <v>43832.625694444447</v>
+      </c>
+      <c r="H28" s="4">
+        <v>49</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M28" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N28" s="4">
+        <v>-89.282340000000005</v>
+      </c>
+      <c r="O28" s="4">
+        <v>13.62866</v>
+      </c>
+      <c r="P28" s="4">
+        <v>315</v>
+      </c>
+      <c r="Q28" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="R28" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="S28" s="4">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C29" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D29" s="4">
+        <v>73220028</v>
+      </c>
+      <c r="E29" s="8">
+        <v>43832.628472222219</v>
+      </c>
+      <c r="F29" s="13">
+        <v>43832.628472222219</v>
+      </c>
+      <c r="G29" s="5">
+        <v>43832.629861111112</v>
+      </c>
+      <c r="H29" s="4">
+        <v>92</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M29" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N29" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="O29" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="P29" s="4">
+        <v>200</v>
+      </c>
+      <c r="Q29" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="R29" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="S29" s="4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C30" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D30" s="4">
+        <v>61305910</v>
+      </c>
+      <c r="E30" s="8">
+        <v>43832.649305555555</v>
+      </c>
+      <c r="F30" s="13">
+        <v>43832.649305555555</v>
+      </c>
+      <c r="G30" s="5">
+        <v>43832.649305555555</v>
+      </c>
+      <c r="H30" s="4">
+        <v>22</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M30" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N30" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="O30" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="P30" s="4">
+        <v>200</v>
+      </c>
+      <c r="Q30" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="R30" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="S30" s="4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C31" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D31" s="4">
+        <v>72424097</v>
+      </c>
+      <c r="E31" s="8">
+        <v>43832.65347222222</v>
+      </c>
+      <c r="F31" s="13">
+        <v>43832.65347222222</v>
+      </c>
+      <c r="G31" s="5">
+        <v>43832.65347222222</v>
+      </c>
+      <c r="H31" s="4">
+        <v>26</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M31" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N31" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="O31" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="P31" s="4">
+        <v>200</v>
+      </c>
+      <c r="Q31" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="R31" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="S31" s="4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C32" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D32" s="4">
+        <v>70017329</v>
+      </c>
+      <c r="E32" s="8">
+        <v>43832.675694444442</v>
+      </c>
+      <c r="F32" s="13">
+        <v>43832.675694444442</v>
+      </c>
+      <c r="G32" s="5">
+        <v>43832.677083333336</v>
+      </c>
+      <c r="H32" s="4">
+        <v>135</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M32" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N32" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="O32" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="P32" s="4">
+        <v>200</v>
+      </c>
+      <c r="Q32" s="4">
+        <v>-89.281000000000006</v>
+      </c>
+      <c r="R32" s="4">
+        <v>13.61547</v>
+      </c>
+      <c r="S32" s="4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C33" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D33" s="4">
+        <v>61305910</v>
+      </c>
+      <c r="E33" s="8">
+        <v>43832.716666666667</v>
+      </c>
+      <c r="F33" s="13">
+        <v>43832.716666666667</v>
+      </c>
+      <c r="G33" s="5">
+        <v>43832.717361111114</v>
+      </c>
+      <c r="H33" s="4">
+        <v>36</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M33" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N33" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="O33" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="P33" s="4">
+        <v>100</v>
+      </c>
+      <c r="Q33" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="R33" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="S33" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C34" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D34" s="4">
+        <v>61305910</v>
+      </c>
+      <c r="E34" s="8">
+        <v>43832.739583333336</v>
+      </c>
+      <c r="F34" s="13">
+        <v>43832.739583333336</v>
+      </c>
+      <c r="G34" s="5">
+        <v>43832.740277777775</v>
+      </c>
+      <c r="H34" s="4">
+        <v>80</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M34" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N34" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="O34" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="P34" s="4">
+        <v>100</v>
+      </c>
+      <c r="Q34" s="4">
+        <v>-89.280910000000006</v>
+      </c>
+      <c r="R34" s="4">
+        <v>13.48343</v>
+      </c>
+      <c r="S34" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C35" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D35" s="4">
+        <v>76589293</v>
+      </c>
+      <c r="E35" s="8">
+        <v>43832.744444444441</v>
+      </c>
+      <c r="F35" s="13">
+        <v>43832.744444444441</v>
+      </c>
+      <c r="G35" s="5">
+        <v>43832.751388888886</v>
+      </c>
+      <c r="H35" s="4">
+        <v>577</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="M35" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N35" s="4">
+        <v>-89.315640000000002</v>
+      </c>
+      <c r="O35" s="4">
+        <v>13.49169</v>
+      </c>
+      <c r="P35" s="4">
+        <v>245</v>
+      </c>
+      <c r="Q35" s="4">
+        <v>-89.308589999999995</v>
+      </c>
+      <c r="R35" s="4">
+        <v>13.516</v>
+      </c>
+      <c r="S35" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C36" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D36" s="4">
+        <v>74408985</v>
+      </c>
+      <c r="E36" s="8">
+        <v>43832.75277777778</v>
+      </c>
+      <c r="F36" s="13">
+        <v>43832.75277777778</v>
+      </c>
+      <c r="G36" s="5">
+        <v>43832.756944444445</v>
+      </c>
+      <c r="H36" s="4">
+        <v>353</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M36" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N36" s="4">
+        <v>-89.293660000000003</v>
+      </c>
+      <c r="O36" s="4">
+        <v>13.54691</v>
+      </c>
+      <c r="P36" s="4">
+        <v>205</v>
+      </c>
+      <c r="Q36" s="4">
+        <v>-89.289699999999996</v>
+      </c>
+      <c r="R36" s="4">
+        <v>13.59155</v>
+      </c>
+      <c r="S36" s="4">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C37" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D37" s="4">
+        <v>70017329</v>
+      </c>
+      <c r="E37" s="8">
+        <v>43832.822222222225</v>
+      </c>
+      <c r="F37" s="13">
+        <v>43832.822222222225</v>
+      </c>
+      <c r="G37" s="5">
+        <v>43832.823611111111</v>
+      </c>
+      <c r="H37" s="4">
+        <v>83</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K37" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="M37" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N37" s="4">
+        <v>-89.282340000000005</v>
+      </c>
+      <c r="O37" s="4">
+        <v>13.62866</v>
+      </c>
+      <c r="P37" s="4">
+        <v>315</v>
+      </c>
+      <c r="Q37" s="4">
+        <v>-89.28989</v>
+      </c>
+      <c r="R37" s="4">
+        <v>13.64878</v>
+      </c>
+      <c r="S37" s="4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B38" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C38" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D38" s="4">
+        <v>70017329</v>
+      </c>
+      <c r="E38" s="8">
+        <v>43832.842361111114</v>
+      </c>
+      <c r="F38" s="13">
+        <v>43832.842361111114</v>
+      </c>
+      <c r="G38" s="5">
+        <v>43832.842361111114</v>
+      </c>
+      <c r="H38" s="4">
+        <v>31</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K38" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M38" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N38" s="4">
+        <v>-89.310249999999996</v>
+      </c>
+      <c r="O38" s="4">
+        <v>13.81606</v>
+      </c>
+      <c r="P38" s="4">
+        <v>240</v>
+      </c>
+      <c r="Q38" s="4">
+        <v>-89.310249999999996</v>
+      </c>
+      <c r="R38" s="4">
+        <v>13.81606</v>
+      </c>
+      <c r="S38" s="4">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B39" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C39" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D39" s="4">
+        <v>74408985</v>
+      </c>
+      <c r="E39" s="8">
+        <v>43832.843055555553</v>
+      </c>
+      <c r="F39" s="13">
+        <v>43832.843055555553</v>
+      </c>
+      <c r="G39" s="5">
+        <v>43832.844444444447</v>
+      </c>
+      <c r="H39" s="4">
+        <v>121</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K39" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M39" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N39" s="4">
+        <v>-89.310249999999996</v>
+      </c>
+      <c r="O39" s="4">
+        <v>13.81606</v>
+      </c>
+      <c r="P39" s="4">
+        <v>80</v>
+      </c>
+      <c r="Q39" s="4">
+        <v>-89.273139</v>
+      </c>
+      <c r="R39" s="4">
+        <v>13.822564</v>
+      </c>
+      <c r="S39" s="4">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B40" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C40" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D40" s="4">
+        <v>74408985</v>
+      </c>
+      <c r="E40" s="8">
+        <v>43832.845138888886</v>
+      </c>
+      <c r="F40" s="13">
+        <v>43832.845138888886</v>
+      </c>
+      <c r="G40" s="5">
+        <v>43832.856944444444</v>
+      </c>
+      <c r="H40" s="4">
+        <v>1054</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M40" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N40" s="4">
+        <v>-89.267319999999998</v>
+      </c>
+      <c r="O40" s="4">
+        <v>13.82892</v>
+      </c>
+      <c r="P40" s="4">
+        <v>250</v>
+      </c>
+      <c r="Q40" s="4">
+        <v>-89.267319999999998</v>
+      </c>
+      <c r="R40" s="4">
+        <v>13.82892</v>
+      </c>
+      <c r="S40" s="4">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C41" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D41" s="4">
+        <v>700</v>
+      </c>
+      <c r="E41" s="8">
+        <v>43832.861805555556</v>
+      </c>
+      <c r="F41" s="13">
+        <v>43832.861805555556</v>
+      </c>
+      <c r="G41" s="5">
+        <v>43832.862500000003</v>
+      </c>
+      <c r="H41" s="4">
+        <v>1</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K41" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M41" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N41" s="4">
+        <v>-89.253429999999994</v>
+      </c>
+      <c r="O41" s="4">
+        <v>13.82132</v>
+      </c>
+      <c r="P41" s="4">
+        <v>120</v>
+      </c>
+      <c r="Q41" s="4">
+        <v>-89.253429999999994</v>
+      </c>
+      <c r="R41" s="4">
+        <v>13.82132</v>
+      </c>
+      <c r="S41" s="4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C42" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D42" s="4">
+        <v>61853812</v>
+      </c>
+      <c r="E42" s="8">
+        <v>43832.893750000003</v>
+      </c>
+      <c r="F42" s="13">
+        <v>43832.893750000003</v>
+      </c>
+      <c r="G42" s="5">
+        <v>43832.893750000003</v>
+      </c>
+      <c r="H42" s="4">
+        <v>22</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J42" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L42" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M42" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N42" s="4">
+        <v>-89.367580000000004</v>
+      </c>
+      <c r="O42" s="4">
+        <v>13.49591</v>
+      </c>
+      <c r="P42" s="4">
+        <v>130</v>
+      </c>
+      <c r="Q42" s="4">
+        <v>-89.367580000000004</v>
+      </c>
+      <c r="R42" s="4">
+        <v>13.49591</v>
+      </c>
+      <c r="S42" s="4">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C43" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D43" s="4">
+        <v>76589293</v>
+      </c>
+      <c r="E43" s="8">
+        <v>43833.422222222223</v>
+      </c>
+      <c r="F43" s="13">
+        <v>43833.422222222223</v>
+      </c>
+      <c r="G43" s="5">
+        <v>43833.422222222223</v>
+      </c>
+      <c r="H43" s="4">
+        <v>14</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K43" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L43" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M43" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N43" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O43" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P43" s="4">
+        <v>50</v>
+      </c>
+      <c r="Q43" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R43" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S43" s="4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C44" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D44" s="4">
+        <v>76589293</v>
+      </c>
+      <c r="E44" s="8">
+        <v>43833.465277777781</v>
+      </c>
+      <c r="F44" s="13">
+        <v>43833.465277777781</v>
+      </c>
+      <c r="G44" s="5">
+        <v>43833.46597222222</v>
+      </c>
+      <c r="H44" s="4">
+        <v>71</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K44" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M44" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N44" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O44" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P44" s="4">
+        <v>50</v>
+      </c>
+      <c r="Q44" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R44" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S44" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C45" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D45" s="4">
+        <v>61619560</v>
+      </c>
+      <c r="E45" s="8">
+        <v>43833.504166666666</v>
+      </c>
+      <c r="F45" s="13">
+        <v>43833.504166666666</v>
+      </c>
+      <c r="G45" s="5">
+        <v>43833.504861111112</v>
+      </c>
+      <c r="H45" s="4">
+        <v>74</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K45" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L45" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M45" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N45" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O45" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P45" s="4">
+        <v>50</v>
+      </c>
+      <c r="Q45" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R45" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S45" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C46" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D46" s="4">
+        <v>60186073</v>
+      </c>
+      <c r="E46" s="8">
+        <v>43833.509027777778</v>
+      </c>
+      <c r="F46" s="13">
+        <v>43833.509027777778</v>
+      </c>
+      <c r="G46" s="5">
+        <v>43833.511805555558</v>
+      </c>
+      <c r="H46" s="4">
+        <v>291</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K46" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L46" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M46" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N46" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O46" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P46" s="4">
+        <v>50</v>
+      </c>
+      <c r="Q46" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R46" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S46" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B47" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C47" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D47" s="4">
+        <v>61619560</v>
+      </c>
+      <c r="E47" s="8">
+        <v>43833.54583333333</v>
+      </c>
+      <c r="F47" s="13">
+        <v>43833.54583333333</v>
+      </c>
+      <c r="G47" s="5">
+        <v>43833.547222222223</v>
+      </c>
+      <c r="H47" s="4">
+        <v>143</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K47" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M47" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N47" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O47" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P47" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q47" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R47" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S47" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A48" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B48" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C48" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D48" s="4">
+        <v>61619560</v>
+      </c>
+      <c r="E48" s="8">
+        <v>43833.61041666667</v>
+      </c>
+      <c r="F48" s="13">
+        <v>43833.61041666667</v>
+      </c>
+      <c r="G48" s="5">
+        <v>43833.613888888889</v>
+      </c>
+      <c r="H48" s="4">
+        <v>308</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K48" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M48" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N48" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O48" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P48" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q48" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R48" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S48" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C49" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D49" s="4">
+        <v>74854632</v>
+      </c>
+      <c r="E49" s="8">
+        <v>43833.620138888888</v>
+      </c>
+      <c r="F49" s="13">
+        <v>43833.620138888888</v>
+      </c>
+      <c r="G49" s="5">
+        <v>43833.620833333334</v>
+      </c>
+      <c r="H49" s="4">
+        <v>30</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K49" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L49" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M49" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N49" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O49" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P49" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q49" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R49" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S49" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B50" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C50" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D50" s="4">
+        <v>61619560</v>
+      </c>
+      <c r="E50" s="8">
+        <v>43833.62222222222</v>
+      </c>
+      <c r="F50" s="13">
+        <v>43833.62222222222</v>
+      </c>
+      <c r="G50" s="5">
+        <v>43833.622916666667</v>
+      </c>
+      <c r="H50" s="4">
+        <v>51</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K50" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M50" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N50" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="O50" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="P50" s="4">
+        <v>175</v>
+      </c>
+      <c r="Q50" s="4">
+        <v>-89.278509999999997</v>
+      </c>
+      <c r="R50" s="4">
+        <v>13.66714</v>
+      </c>
+      <c r="S50" s="4">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B51" s="4">
+        <v>61090192</v>
+      </c>
+      <c r="C51" s="11">
+        <v>860766049463800</v>
+      </c>
+      <c r="D51" s="4">
+        <v>72470704</v>
+      </c>
+      <c r="E51" s="8">
+        <v>43833.691666666666</v>
+      </c>
+      <c r="F51" s="13">
+        <v>43833.691666666666</v>
+      </c>
+      <c r="G51" s="5">
+        <v>43833.692361111112</v>
+      </c>
+      <c r="H51" s="4">
+        <v>44</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="K51" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="L51" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="M51" s="11">
+        <v>706040000000000</v>
+      </c>
+      <c r="N51" s="4">
+        <v>-89.289249999999996</v>
+      </c>
+      <c r="O51" s="4">
+        <v>13.671580000000001</v>
+      </c>
+      <c r="P51" s="4">
+        <v>10</v>
+      </c>
+      <c r="Q51" s="4">
+        <v>-89.289249999999996</v>
+      </c>
+      <c r="R51" s="4">
+        <v>13.671580000000001</v>
+      </c>
+      <c r="S51" s="4">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>